<commit_message>
script que sobe regionais novas
</commit_message>
<xml_diff>
--- a/proposta mudanças e nova regional.xlsx
+++ b/proposta mudanças e nova regional.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sesibahia-my.sharepoint.com/personal/jorge_sm_fieb_org_br/Documents/Documentos/Observatorio/FIEB/Regionais/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="11_F6E6CF92C9E748091061005C784339F02100AF73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6837FC04-E7DF-4BE3-934C-1DFADB5B0358}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="11_F6E6CF92C9E748091061005C784339F02100AF73" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DD08C14-DFE9-42E1-A389-B35B98407EBC}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-2010" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -1447,13 +1447,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{15F798F4-7531-42E0-AF0E-27ADF195FAD7}" name="Tabela3" displayName="Tabela3" ref="A1:F418" totalsRowShown="0">
-  <autoFilter ref="A1:F418" xr:uid="{15F798F4-7531-42E0-AF0E-27ADF195FAD7}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="SEABRA"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F418" xr:uid="{15F798F4-7531-42E0-AF0E-27ADF195FAD7}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{E9385C55-71CE-4EDB-AFD5-459D70E25F42}" name="NO_TERRITORIO"/>
     <tableColumn id="2" xr3:uid="{582F5846-64C2-4F1E-A99B-93981A6F1018}" name="NO_MUNICIPIO"/>
@@ -1814,7 +1808,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1834,7 +1828,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1851,7 +1845,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1868,7 +1862,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1885,7 +1879,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1902,7 +1896,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1919,7 +1913,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1936,7 +1930,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1953,7 +1947,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1970,7 +1964,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1987,7 +1981,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -2004,7 +1998,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -2021,7 +2015,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -2038,7 +2032,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -2058,7 +2052,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -2075,7 +2069,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -2092,7 +2086,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -2109,7 +2103,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -2126,7 +2120,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -2143,7 +2137,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -2160,7 +2154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -2177,7 +2171,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -2194,7 +2188,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -2211,7 +2205,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -2228,7 +2222,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -2245,7 +2239,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -2262,7 +2256,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2279,7 +2273,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -2296,7 +2290,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -2313,7 +2307,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -2330,7 +2324,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>54</v>
       </c>
@@ -2347,7 +2341,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -2364,7 +2358,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>57</v>
       </c>
@@ -2381,7 +2375,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -2401,7 +2395,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>30</v>
       </c>
@@ -2418,7 +2412,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -2435,7 +2429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>16</v>
       </c>
@@ -2452,7 +2446,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>35</v>
       </c>
@@ -2469,7 +2463,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -2486,7 +2480,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>22</v>
       </c>
@@ -2503,7 +2497,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -2520,7 +2514,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>67</v>
       </c>
@@ -2537,7 +2531,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>30</v>
       </c>
@@ -2554,7 +2548,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>46</v>
       </c>
@@ -2571,7 +2565,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -2588,7 +2582,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>72</v>
       </c>
@@ -2605,7 +2599,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>57</v>
       </c>
@@ -2622,7 +2616,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -2639,7 +2633,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>2</v>
       </c>
@@ -2659,7 +2653,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>2</v>
       </c>
@@ -2679,7 +2673,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>78</v>
       </c>
@@ -2696,7 +2690,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>78</v>
       </c>
@@ -2713,7 +2707,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>25</v>
       </c>
@@ -2730,7 +2724,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>82</v>
       </c>
@@ -2747,7 +2741,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>57</v>
       </c>
@@ -2764,7 +2758,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>85</v>
       </c>
@@ -2781,7 +2775,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>22</v>
       </c>
@@ -2798,7 +2792,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>35</v>
       </c>
@@ -2815,7 +2809,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>89</v>
       </c>
@@ -2832,7 +2826,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>91</v>
       </c>
@@ -2849,7 +2843,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>91</v>
       </c>
@@ -2866,7 +2860,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>85</v>
       </c>
@@ -2883,7 +2877,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>95</v>
       </c>
@@ -2900,7 +2894,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>30</v>
       </c>
@@ -2917,7 +2911,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>85</v>
       </c>
@@ -2934,7 +2928,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>28</v>
       </c>
@@ -2951,7 +2945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>50</v>
       </c>
@@ -2968,7 +2962,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>33</v>
       </c>
@@ -2985,7 +2979,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>22</v>
       </c>
@@ -3002,7 +2996,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>103</v>
       </c>
@@ -3022,7 +3016,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>50</v>
       </c>
@@ -3039,7 +3033,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>106</v>
       </c>
@@ -3056,7 +3050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>33</v>
       </c>
@@ -3073,7 +3067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>82</v>
       </c>
@@ -3090,7 +3084,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>28</v>
       </c>
@@ -3107,7 +3101,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>22</v>
       </c>
@@ -3124,7 +3118,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>46</v>
       </c>
@@ -3141,7 +3135,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>103</v>
       </c>
@@ -3158,7 +3152,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>85</v>
       </c>
@@ -3175,7 +3169,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>30</v>
       </c>
@@ -3192,7 +3186,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>46</v>
       </c>
@@ -3209,7 +3203,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>106</v>
       </c>
@@ -3226,7 +3220,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>54</v>
       </c>
@@ -3243,7 +3237,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>54</v>
       </c>
@@ -3260,7 +3254,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>30</v>
       </c>
@@ -3277,7 +3271,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>20</v>
       </c>
@@ -3294,7 +3288,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -3311,7 +3305,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>57</v>
       </c>
@@ -3328,7 +3322,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>106</v>
       </c>
@@ -3345,7 +3339,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>91</v>
       </c>
@@ -3362,7 +3356,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>35</v>
       </c>
@@ -3379,7 +3373,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -3396,7 +3390,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>78</v>
       </c>
@@ -3413,7 +3407,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>28</v>
       </c>
@@ -3430,7 +3424,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>6</v>
       </c>
@@ -3447,7 +3441,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>12</v>
       </c>
@@ -3464,7 +3458,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>12</v>
       </c>
@@ -3481,7 +3475,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>22</v>
       </c>
@@ -3498,7 +3492,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>82</v>
       </c>
@@ -3515,7 +3509,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>14</v>
       </c>
@@ -3532,7 +3526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>91</v>
       </c>
@@ -3549,7 +3543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>46</v>
       </c>
@@ -3566,7 +3560,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>14</v>
       </c>
@@ -3583,7 +3577,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>8</v>
       </c>
@@ -3600,7 +3594,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>30</v>
       </c>
@@ -3617,7 +3611,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>85</v>
       </c>
@@ -3634,7 +3628,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>14</v>
       </c>
@@ -3651,7 +3645,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>30</v>
       </c>
@@ -3668,7 +3662,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>82</v>
       </c>
@@ -3685,7 +3679,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>12</v>
       </c>
@@ -3702,7 +3696,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>82</v>
       </c>
@@ -3719,7 +3713,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>35</v>
       </c>
@@ -3736,7 +3730,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>25</v>
       </c>
@@ -3753,7 +3747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>8</v>
       </c>
@@ -3770,7 +3764,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>35</v>
       </c>
@@ -3787,7 +3781,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>91</v>
       </c>
@@ -3804,7 +3798,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>106</v>
       </c>
@@ -3821,7 +3815,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>16</v>
       </c>
@@ -3838,7 +3832,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>103</v>
       </c>
@@ -3855,7 +3849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>85</v>
       </c>
@@ -3872,7 +3866,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>91</v>
       </c>
@@ -3889,7 +3883,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>25</v>
       </c>
@@ -3906,7 +3900,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>30</v>
       </c>
@@ -3923,7 +3917,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>8</v>
       </c>
@@ -3940,7 +3934,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>78</v>
       </c>
@@ -3957,7 +3951,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>8</v>
       </c>
@@ -3974,7 +3968,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>12</v>
       </c>
@@ -3991,7 +3985,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>67</v>
       </c>
@@ -4008,7 +4002,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>12</v>
       </c>
@@ -4025,7 +4019,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>57</v>
       </c>
@@ -4042,7 +4036,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>14</v>
       </c>
@@ -4059,7 +4053,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>33</v>
       </c>
@@ -4076,7 +4070,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>89</v>
       </c>
@@ -4093,7 +4087,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>22</v>
       </c>
@@ -4110,7 +4104,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>35</v>
       </c>
@@ -4127,7 +4121,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>50</v>
       </c>
@@ -4144,7 +4138,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>54</v>
       </c>
@@ -4161,7 +4155,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>28</v>
       </c>
@@ -4178,7 +4172,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>6</v>
       </c>
@@ -4195,7 +4189,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>16</v>
       </c>
@@ -4212,7 +4206,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>91</v>
       </c>
@@ -4229,7 +4223,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>30</v>
       </c>
@@ -4246,7 +4240,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>85</v>
       </c>
@@ -4263,7 +4257,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>67</v>
       </c>
@@ -4280,7 +4274,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>12</v>
       </c>
@@ -4297,7 +4291,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>72</v>
       </c>
@@ -4314,7 +4308,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="148" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>85</v>
       </c>
@@ -4331,7 +4325,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>22</v>
       </c>
@@ -4348,7 +4342,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>2</v>
       </c>
@@ -4368,7 +4362,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>89</v>
       </c>
@@ -4385,7 +4379,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>28</v>
       </c>
@@ -4402,7 +4396,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>78</v>
       </c>
@@ -4419,7 +4413,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>72</v>
       </c>
@@ -4436,7 +4430,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>50</v>
       </c>
@@ -4453,7 +4447,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>20</v>
       </c>
@@ -4470,7 +4464,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>16</v>
       </c>
@@ -4487,7 +4481,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>2</v>
       </c>
@@ -4507,7 +4501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>28</v>
       </c>
@@ -4524,7 +4518,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>57</v>
       </c>
@@ -4541,7 +4535,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>46</v>
       </c>
@@ -4558,7 +4552,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="162" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>57</v>
       </c>
@@ -4575,7 +4569,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="163" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>50</v>
       </c>
@@ -4592,7 +4586,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>89</v>
       </c>
@@ -4609,7 +4603,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="165" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>22</v>
       </c>
@@ -4626,7 +4620,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>8</v>
       </c>
@@ -4643,7 +4637,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>14</v>
       </c>
@@ -4660,7 +4654,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>16</v>
       </c>
@@ -4677,7 +4671,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>54</v>
       </c>
@@ -4694,7 +4688,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>28</v>
       </c>
@@ -4711,7 +4705,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="171" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>25</v>
       </c>
@@ -4728,7 +4722,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="172" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>25</v>
       </c>
@@ -4745,7 +4739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="173" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>2</v>
       </c>
@@ -4765,7 +4759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="174" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>14</v>
       </c>
@@ -4782,7 +4776,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>28</v>
       </c>
@@ -4799,7 +4793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>67</v>
       </c>
@@ -4816,7 +4810,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>72</v>
       </c>
@@ -4833,7 +4827,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>22</v>
       </c>
@@ -4850,7 +4844,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>22</v>
       </c>
@@ -4867,7 +4861,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="180" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>2</v>
       </c>
@@ -4887,7 +4881,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>16</v>
       </c>
@@ -4904,7 +4898,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>16</v>
       </c>
@@ -4921,7 +4915,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="183" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>67</v>
       </c>
@@ -4938,7 +4932,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="184" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>28</v>
       </c>
@@ -4955,7 +4949,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="185" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>22</v>
       </c>
@@ -4972,7 +4966,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="186" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>22</v>
       </c>
@@ -4989,7 +4983,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="187" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>20</v>
       </c>
@@ -5006,7 +5000,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="188" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>16</v>
       </c>
@@ -5023,7 +5017,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="189" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>89</v>
       </c>
@@ -5040,7 +5034,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="190" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>8</v>
       </c>
@@ -5057,7 +5051,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="191" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>20</v>
       </c>
@@ -5074,7 +5068,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="192" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>103</v>
       </c>
@@ -5091,7 +5085,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>22</v>
       </c>
@@ -5108,7 +5102,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>67</v>
       </c>
@@ -5125,7 +5119,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>89</v>
       </c>
@@ -5142,7 +5136,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>8</v>
       </c>
@@ -5159,7 +5153,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>22</v>
       </c>
@@ -5176,7 +5170,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>25</v>
       </c>
@@ -5193,7 +5187,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>89</v>
       </c>
@@ -5210,7 +5204,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>72</v>
       </c>
@@ -5227,7 +5221,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>25</v>
       </c>
@@ -5244,7 +5238,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>46</v>
       </c>
@@ -5261,7 +5255,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>89</v>
       </c>
@@ -5278,7 +5272,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>85</v>
       </c>
@@ -5295,7 +5289,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="205" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>50</v>
       </c>
@@ -5312,7 +5306,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>85</v>
       </c>
@@ -5329,7 +5323,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>82</v>
       </c>
@@ -5346,7 +5340,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="208" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>30</v>
       </c>
@@ -5363,7 +5357,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="209" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>95</v>
       </c>
@@ -5380,7 +5374,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="210" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>25</v>
       </c>
@@ -5397,7 +5391,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="211" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>33</v>
       </c>
@@ -5414,7 +5408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="212" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>50</v>
       </c>
@@ -5431,7 +5425,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="213" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>8</v>
       </c>
@@ -5448,7 +5442,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="214" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>16</v>
       </c>
@@ -5465,7 +5459,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="215" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>12</v>
       </c>
@@ -5482,7 +5476,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="216" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>25</v>
       </c>
@@ -5499,7 +5493,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="217" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>16</v>
       </c>
@@ -5516,7 +5510,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="218" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>28</v>
       </c>
@@ -5533,7 +5527,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="219" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>106</v>
       </c>
@@ -5550,7 +5544,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="220" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>20</v>
       </c>
@@ -5567,7 +5561,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="221" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>28</v>
       </c>
@@ -5584,7 +5578,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="222" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>22</v>
       </c>
@@ -5601,7 +5595,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="223" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>2</v>
       </c>
@@ -5621,7 +5615,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>25</v>
       </c>
@@ -5638,7 +5632,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="225" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>85</v>
       </c>
@@ -5655,7 +5649,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="226" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>25</v>
       </c>
@@ -5672,7 +5666,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>20</v>
       </c>
@@ -5689,7 +5683,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="228" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>72</v>
       </c>
@@ -5706,7 +5700,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="229" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>25</v>
       </c>
@@ -5723,7 +5717,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="230" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>46</v>
       </c>
@@ -5740,7 +5734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="231" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>28</v>
       </c>
@@ -5757,7 +5751,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="232" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>103</v>
       </c>
@@ -5774,7 +5768,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="233" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>2</v>
       </c>
@@ -5794,7 +5788,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="234" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>30</v>
       </c>
@@ -5811,7 +5805,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="235" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>85</v>
       </c>
@@ -5828,7 +5822,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="236" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>35</v>
       </c>
@@ -5845,7 +5839,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="237" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>72</v>
       </c>
@@ -5862,7 +5856,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="238" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>89</v>
       </c>
@@ -5879,7 +5873,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="239" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>78</v>
       </c>
@@ -5896,7 +5890,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="240" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>6</v>
       </c>
@@ -5913,7 +5907,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="241" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>103</v>
       </c>
@@ -5930,7 +5924,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="242" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>30</v>
       </c>
@@ -5947,7 +5941,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="243" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>89</v>
       </c>
@@ -5964,7 +5958,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="244" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>54</v>
       </c>
@@ -5981,7 +5975,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="245" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>57</v>
       </c>
@@ -5998,7 +5992,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>85</v>
       </c>
@@ -6015,7 +6009,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="247" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>16</v>
       </c>
@@ -6032,7 +6026,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="248" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>35</v>
       </c>
@@ -6049,7 +6043,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="249" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>25</v>
       </c>
@@ -6066,7 +6060,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="250" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>91</v>
       </c>
@@ -6083,7 +6077,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="251" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>22</v>
       </c>
@@ -6100,7 +6094,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="252" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>2</v>
       </c>
@@ -6120,7 +6114,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>22</v>
       </c>
@@ -6137,7 +6131,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="254" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>103</v>
       </c>
@@ -6154,7 +6148,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="255" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>57</v>
       </c>
@@ -6171,7 +6165,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="256" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>20</v>
       </c>
@@ -6188,7 +6182,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="257" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>95</v>
       </c>
@@ -6205,7 +6199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="258" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>25</v>
       </c>
@@ -6222,7 +6216,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="259" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>95</v>
       </c>
@@ -6239,7 +6233,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="260" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>30</v>
       </c>
@@ -6256,7 +6250,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="261" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>46</v>
       </c>
@@ -6273,7 +6267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="262" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>57</v>
       </c>
@@ -6290,7 +6284,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="263" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>2</v>
       </c>
@@ -6310,7 +6304,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>30</v>
       </c>
@@ -6327,7 +6321,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="265" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>2</v>
       </c>
@@ -6347,7 +6341,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="266" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>20</v>
       </c>
@@ -6364,7 +6358,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="267" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>28</v>
       </c>
@@ -6381,7 +6375,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="268" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>72</v>
       </c>
@@ -6398,7 +6392,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="269" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>91</v>
       </c>
@@ -6415,7 +6409,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="270" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>57</v>
       </c>
@@ -6432,7 +6426,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="271" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>91</v>
       </c>
@@ -6449,7 +6443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="272" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>25</v>
       </c>
@@ -6466,7 +6460,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="273" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>91</v>
       </c>
@@ -6483,7 +6477,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="274" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>50</v>
       </c>
@@ -6500,7 +6494,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="275" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>46</v>
       </c>
@@ -6517,7 +6511,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="276" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>89</v>
       </c>
@@ -6534,7 +6528,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="277" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>54</v>
       </c>
@@ -6551,7 +6545,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="278" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>16</v>
       </c>
@@ -6568,7 +6562,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="279" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>25</v>
       </c>
@@ -6585,7 +6579,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="280" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>2</v>
       </c>
@@ -6605,7 +6599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="281" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>12</v>
       </c>
@@ -6622,7 +6616,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="282" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>20</v>
       </c>
@@ -6639,7 +6633,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="283" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>2</v>
       </c>
@@ -6659,7 +6653,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="284" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>12</v>
       </c>
@@ -6676,7 +6670,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="285" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>8</v>
       </c>
@@ -6693,7 +6687,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="286" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>57</v>
       </c>
@@ -6710,7 +6704,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="287" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>8</v>
       </c>
@@ -6727,7 +6721,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="288" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>95</v>
       </c>
@@ -6744,7 +6738,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="289" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>85</v>
       </c>
@@ -6761,7 +6755,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="290" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>2</v>
       </c>
@@ -6781,7 +6775,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="291" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>78</v>
       </c>
@@ -6798,7 +6792,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="292" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>57</v>
       </c>
@@ -6815,7 +6809,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="293" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>12</v>
       </c>
@@ -6832,7 +6826,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="294" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>22</v>
       </c>
@@ -6849,7 +6843,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="295" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>6</v>
       </c>
@@ -6866,7 +6860,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="296" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>54</v>
       </c>
@@ -6883,7 +6877,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="297" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>8</v>
       </c>
@@ -6900,7 +6894,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="298" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>12</v>
       </c>
@@ -6917,7 +6911,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="299" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>2</v>
       </c>
@@ -6937,7 +6931,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="300" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>106</v>
       </c>
@@ -6954,7 +6948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="301" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>85</v>
       </c>
@@ -6971,7 +6965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="302" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>33</v>
       </c>
@@ -6988,7 +6982,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="303" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>54</v>
       </c>
@@ -7005,7 +6999,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="304" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>50</v>
       </c>
@@ -7022,7 +7016,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="305" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>30</v>
       </c>
@@ -7039,7 +7033,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="306" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>72</v>
       </c>
@@ -7056,7 +7050,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="307" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>25</v>
       </c>
@@ -7073,7 +7067,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>30</v>
       </c>
@@ -7090,7 +7084,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="309" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>30</v>
       </c>
@@ -7107,7 +7101,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="310" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>103</v>
       </c>
@@ -7124,7 +7118,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="311" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>33</v>
       </c>
@@ -7141,7 +7135,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="312" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>67</v>
       </c>
@@ -7158,7 +7152,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="313" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>89</v>
       </c>
@@ -7175,7 +7169,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>20</v>
       </c>
@@ -7192,7 +7186,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="315" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>28</v>
       </c>
@@ -7209,7 +7203,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="316" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>30</v>
       </c>
@@ -7226,7 +7220,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="317" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>50</v>
       </c>
@@ -7243,7 +7237,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>46</v>
       </c>
@@ -7260,7 +7254,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="319" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>46</v>
       </c>
@@ -7277,7 +7271,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="320" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>54</v>
       </c>
@@ -7294,7 +7288,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="321" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>72</v>
       </c>
@@ -7311,7 +7305,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="322" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>106</v>
       </c>
@@ -7328,7 +7322,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="323" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>46</v>
       </c>
@@ -7345,7 +7339,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="324" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>35</v>
       </c>
@@ -7362,7 +7356,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="325" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>54</v>
       </c>
@@ -7379,7 +7373,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="326" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>57</v>
       </c>
@@ -7396,7 +7390,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="327" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>12</v>
       </c>
@@ -7413,7 +7407,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="328" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>12</v>
       </c>
@@ -7430,7 +7424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="329" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>30</v>
       </c>
@@ -7447,7 +7441,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="330" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>2</v>
       </c>
@@ -7467,7 +7461,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="331" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>85</v>
       </c>
@@ -7484,7 +7478,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="332" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>78</v>
       </c>
@@ -7501,7 +7495,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="333" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>8</v>
       </c>
@@ -7518,7 +7512,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="334" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>6</v>
       </c>
@@ -7535,7 +7529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="335" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>72</v>
       </c>
@@ -7552,7 +7546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="336" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>91</v>
       </c>
@@ -7569,7 +7563,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="337" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>103</v>
       </c>
@@ -7586,7 +7580,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="338" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>14</v>
       </c>
@@ -7603,7 +7597,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="339" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>12</v>
       </c>
@@ -7620,7 +7614,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="340" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>67</v>
       </c>
@@ -7637,7 +7631,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="341" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>89</v>
       </c>
@@ -7654,7 +7648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="342" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>25</v>
       </c>
@@ -7671,7 +7665,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="343" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>22</v>
       </c>
@@ -7688,7 +7682,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="344" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>82</v>
       </c>
@@ -7705,7 +7699,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="345" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>35</v>
       </c>
@@ -7722,7 +7716,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="346" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>72</v>
       </c>
@@ -7739,7 +7733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="347" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>46</v>
       </c>
@@ -7756,7 +7750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="348" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>82</v>
       </c>
@@ -7773,7 +7767,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="349" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>14</v>
       </c>
@@ -7790,7 +7784,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="350" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>91</v>
       </c>
@@ -7807,7 +7801,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="351" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>91</v>
       </c>
@@ -7824,7 +7818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="352" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>14</v>
       </c>
@@ -7841,7 +7835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="353" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>35</v>
       </c>
@@ -7858,7 +7852,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="354" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>46</v>
       </c>
@@ -7875,7 +7869,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="355" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>91</v>
       </c>
@@ -7892,7 +7886,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="356" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>91</v>
       </c>
@@ -7909,7 +7903,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="357" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>82</v>
       </c>
@@ -7926,7 +7920,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="358" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>103</v>
       </c>
@@ -7943,7 +7937,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="359" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>28</v>
       </c>
@@ -7960,7 +7954,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="360" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>14</v>
       </c>
@@ -7977,7 +7971,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="361" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>22</v>
       </c>
@@ -7994,7 +7988,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="362" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>54</v>
       </c>
@@ -8011,7 +8005,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="363" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>25</v>
       </c>
@@ -8028,7 +8022,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="364" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>103</v>
       </c>
@@ -8045,7 +8039,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="365" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>91</v>
       </c>
@@ -8062,7 +8056,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="366" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>8</v>
       </c>
@@ -8079,7 +8073,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="367" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>91</v>
       </c>
@@ -8096,7 +8090,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="368" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>95</v>
       </c>
@@ -8133,7 +8127,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="370" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>85</v>
       </c>
@@ -8150,7 +8144,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="371" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>33</v>
       </c>
@@ -8167,7 +8161,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="372" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>106</v>
       </c>
@@ -8184,7 +8178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="373" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>57</v>
       </c>
@@ -8201,7 +8195,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="374" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>82</v>
       </c>
@@ -8218,7 +8212,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="375" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>54</v>
       </c>
@@ -8235,7 +8229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="376" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>46</v>
       </c>
@@ -8252,7 +8246,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="377" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>95</v>
       </c>
@@ -8269,7 +8263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="378" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>103</v>
       </c>
@@ -8286,7 +8280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="379" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>57</v>
       </c>
@@ -8303,7 +8297,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="380" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>12</v>
       </c>
@@ -8320,7 +8314,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="381" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>106</v>
       </c>
@@ -8337,7 +8331,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="382" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>2</v>
       </c>
@@ -8357,7 +8351,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="383" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>82</v>
       </c>
@@ -8374,7 +8368,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="384" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>85</v>
       </c>
@@ -8391,7 +8385,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="385" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>85</v>
       </c>
@@ -8408,7 +8402,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="386" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>14</v>
       </c>
@@ -8425,7 +8419,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="387" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>50</v>
       </c>
@@ -8442,7 +8436,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="388" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>72</v>
       </c>
@@ -8459,7 +8453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="389" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>20</v>
       </c>
@@ -8476,7 +8470,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="390" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>14</v>
       </c>
@@ -8493,7 +8487,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="391" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>46</v>
       </c>
@@ -8510,7 +8504,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="392" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>50</v>
       </c>
@@ -8527,7 +8521,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="393" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>14</v>
       </c>
@@ -8544,7 +8538,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="394" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>30</v>
       </c>
@@ -8561,7 +8555,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="395" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>46</v>
       </c>
@@ -8578,7 +8572,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="396" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>106</v>
       </c>
@@ -8595,7 +8589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="397" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>25</v>
       </c>
@@ -8612,7 +8606,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="398" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>22</v>
       </c>
@@ -8629,7 +8623,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="399" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>16</v>
       </c>
@@ -8646,7 +8640,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="400" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>28</v>
       </c>
@@ -8663,7 +8657,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="401" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>95</v>
       </c>
@@ -8680,7 +8674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="402" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>22</v>
       </c>
@@ -8697,7 +8691,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="403" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>85</v>
       </c>
@@ -8714,7 +8708,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="404" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>22</v>
       </c>
@@ -8731,7 +8725,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="405" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>2</v>
       </c>
@@ -8751,7 +8745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="406" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>50</v>
       </c>
@@ -8768,7 +8762,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="407" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>46</v>
       </c>
@@ -8785,7 +8779,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="408" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>54</v>
       </c>
@@ -8802,7 +8796,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="409" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
         <v>54</v>
       </c>
@@ -8819,7 +8813,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="410" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A410" t="s">
         <v>95</v>
       </c>
@@ -8836,7 +8830,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="411" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A411" t="s">
         <v>91</v>
       </c>
@@ -8853,7 +8847,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="412" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>103</v>
       </c>
@@ -8870,7 +8864,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="413" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
         <v>20</v>
       </c>
@@ -8887,7 +8881,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="414" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
         <v>30</v>
       </c>
@@ -8904,7 +8898,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="415" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>2</v>
       </c>
@@ -8924,7 +8918,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="416" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>35</v>
       </c>
@@ -8941,7 +8935,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="417" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>50</v>
       </c>
@@ -8958,7 +8952,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="418" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>28</v>
       </c>

</xml_diff>